<commit_message>
added all the variables to the input sheet
</commit_message>
<xml_diff>
--- a/rpy_input_parameters.xlsx
+++ b/rpy_input_parameters.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samjo\Desktop\clubs\soar\irec_27\controls_eecs\IREC_26-27_Controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C48AE657-A0DF-47D6-A589-8A0482EA3E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2118999-272C-45AE-9A58-8D3226F09276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3850124B-4C10-4519-AB6D-3AC4B4A0B5D5}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" firstSheet="4" activeTab="6" xr2:uid="{3850124B-4C10-4519-AB6D-3AC4B4A0B5D5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Solid Motor" sheetId="1" r:id="rId1"/>
-    <sheet name="Environment" sheetId="2" r:id="rId2"/>
+    <sheet name="Environment" sheetId="2" r:id="rId1"/>
+    <sheet name="Solid Motor" sheetId="1" r:id="rId2"/>
     <sheet name="Rocket" sheetId="3" r:id="rId3"/>
-    <sheet name="Flight" sheetId="4" r:id="rId4"/>
+    <sheet name="Nosecone" sheetId="4" r:id="rId4"/>
+    <sheet name="Trapezoidal Fins" sheetId="5" r:id="rId5"/>
+    <sheet name="Tail" sheetId="6" r:id="rId6"/>
+    <sheet name="Rail Buttons" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="64">
   <si>
     <t>Variable</t>
   </si>
@@ -57,16 +60,199 @@
   </si>
   <si>
     <t>Step</t>
+  </si>
+  <si>
+    <t>thrust_source</t>
+  </si>
+  <si>
+    <t>"AeroTech_M1939W.eng"</t>
+  </si>
+  <si>
+    <t>nozzle_radius</t>
+  </si>
+  <si>
+    <t>grain_number</t>
+  </si>
+  <si>
+    <t>grain_density</t>
+  </si>
+  <si>
+    <t>grain_outer_radius</t>
+  </si>
+  <si>
+    <t>grain_initial_inner_radius</t>
+  </si>
+  <si>
+    <t>grain_initial_height</t>
+  </si>
+  <si>
+    <t>grain_separation</t>
+  </si>
+  <si>
+    <t>grains_center_of_mass_position</t>
+  </si>
+  <si>
+    <t>center_of_dry_mass_position</t>
+  </si>
+  <si>
+    <t>nozzle_position</t>
+  </si>
+  <si>
+    <t>burn_time</t>
+  </si>
+  <si>
+    <t>throat_radius</t>
+  </si>
+  <si>
+    <t>coordinate_system_orientation</t>
+  </si>
+  <si>
+    <t>"nozzle_to_combustion_chamber"</t>
+  </si>
+  <si>
+    <t>dry_inertia_i11</t>
+  </si>
+  <si>
+    <t>dry_inertia_i33</t>
+  </si>
+  <si>
+    <t>dry_inertia_i22</t>
+  </si>
+  <si>
+    <t>radius</t>
+  </si>
+  <si>
+    <t>mass</t>
+  </si>
+  <si>
+    <t>inertia</t>
+  </si>
+  <si>
+    <t>power_off_drag</t>
+  </si>
+  <si>
+    <t>power_on_drag</t>
+  </si>
+  <si>
+    <t>center_of_mass_without_motor</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>tuple</t>
+  </si>
+  <si>
+    <t>"tail_to_nose"</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>length</t>
+  </si>
+  <si>
+    <t>position</t>
+  </si>
+  <si>
+    <t>kind</t>
+  </si>
+  <si>
+    <t>bluffness</t>
+  </si>
+  <si>
+    <t>ogive</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>root_chord</t>
+  </si>
+  <si>
+    <t>tip_chord</t>
+  </si>
+  <si>
+    <t>span</t>
+  </si>
+  <si>
+    <t>rocket_radius</t>
+  </si>
+  <si>
+    <t>sweep_length</t>
+  </si>
+  <si>
+    <t>sweep_angle</t>
+  </si>
+  <si>
+    <t>airfoil</t>
+  </si>
+  <si>
+    <t>base_radius</t>
+  </si>
+  <si>
+    <t>power</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>needed for ogive</t>
+  </si>
+  <si>
+    <t>optional/no impact</t>
+  </si>
+  <si>
+    <t>optional</t>
+  </si>
+  <si>
+    <t>dry_mass</t>
+  </si>
+  <si>
+    <t>reshape_thrust_curve</t>
+  </si>
+  <si>
+    <t>no idea</t>
+  </si>
+  <si>
+    <t>interpolation_method</t>
+  </si>
+  <si>
+    <t>reference_pressure</t>
+  </si>
+  <si>
+    <t>only_radial_burn</t>
+  </si>
+  <si>
+    <t>top_radius</t>
+  </si>
+  <si>
+    <t>bottom_radius</t>
+  </si>
+  <si>
+    <t>upper_button_position</t>
+  </si>
+  <si>
+    <t>lower_button_position</t>
+  </si>
+  <si>
+    <t>angular_position</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -109,20 +295,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A603778A-0AC4-41BA-9377-94967C480B7A}" name="Table2" displayName="Table2" ref="A1:E6" totalsRowShown="0">
-  <autoFilter ref="A1:E6" xr:uid="{A603778A-0AC4-41BA-9377-94967C480B7A}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{90F1D158-6800-491B-9308-9F2FA4C9636B}" name="Variable"/>
-    <tableColumn id="2" xr3:uid="{2563A4CE-ABE0-4CC1-9C84-B63FE4070657}" name="Set"/>
-    <tableColumn id="3" xr3:uid="{E5DD798D-7B61-4CA9-B242-BE9A2C36E575}" name="Min"/>
-    <tableColumn id="5" xr3:uid="{D7D33127-27F0-46FD-8887-46AAA2924181}" name="Max"/>
-    <tableColumn id="4" xr3:uid="{DD275900-F114-4B3A-81E2-6C166B506699}" name="Step"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -441,50 +613,348 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8160EB66-A072-414B-B1B5-A2EF0AE3FFBA}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0D88883-570E-48D5-9EA0-8E8B677054BE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0D88883-570E-48D5-9EA0-8E8B677054BE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8160EB66-A072-414B-B1B5-A2EF0AE3FFBA}">
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <f>(1.75/2) / 39.37</f>
+        <v>2.2225044450088903E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4">
+        <v>3.2690000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5">
+        <f>(1/12)*B4*(3*((0.098/2)*2)+POWER(0.732,2))</f>
+        <v>0.22605788799999998</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6">
+        <f>(1/12)*B4*(3*((0.098/2)*2)+POWER(0.732,2))</f>
+        <v>0.22605788799999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <f>0.5*B4*POWER((0.098/2),2)</f>
+        <v>3.9244345000000007E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <f>0.06576*27679.90471</f>
+        <v>1820.2305337296</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <f>3.365/2/39.37</f>
+        <v>4.2735585471170949E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <f>1.125/2/39.37</f>
+        <v>1.428752857505715E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <f>6/2/39.37</f>
+        <v>7.620015240030481E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <f>6/2/39.37/2</f>
+        <v>3.8100076200152405E-2</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <f>0.732/2</f>
+        <v>0.36599999999999999</v>
+      </c>
+      <c r="D15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+      <c r="D16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <f>0.734/2/39.37</f>
+        <v>9.3218186436372884E-3</v>
+      </c>
+      <c r="D18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DE46F10-F7E4-4FF9-9DF9-CA245AB9C3B3}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2">
+        <f>6.17/2/39.37</f>
+        <v>7.8359156718313436E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>35</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D4D93E-62F8-4675-8413-8C8F2B28BDDF}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="11" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="11" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -500,11 +970,269 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" t="s">
+        <v>51</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C6CA8B0-88A8-433F-A0FC-EB53EF89F6DB}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6">
+        <f>6.17/2/39.37</f>
+        <v>7.8359156718313436E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C24AA439-E62A-4D19-BE31-DD01D82FC1DB}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B40BE1E-2C0B-4286-A3FB-3C7826FF8F5E}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added first set of inputs parsing for solid motors, environment, and rocket. Should be easy to finish now. works, but works like shit.
</commit_message>
<xml_diff>
--- a/rpy_input_parameters.xlsx
+++ b/rpy_input_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samjo\Desktop\clubs\soar\irec_27\controls_eecs\IREC_26-27_Controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2118999-272C-45AE-9A58-8D3226F09276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A6356C-3C7C-4424-9938-772D6081D2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" firstSheet="4" activeTab="6" xr2:uid="{3850124B-4C10-4519-AB6D-3AC4B4A0B5D5}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{3850124B-4C10-4519-AB6D-3AC4B4A0B5D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Environment" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="78">
   <si>
     <t>Variable</t>
   </si>
@@ -65,9 +65,6 @@
     <t>thrust_source</t>
   </si>
   <si>
-    <t>"AeroTech_M1939W.eng"</t>
-  </si>
-  <si>
     <t>nozzle_radius</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>coordinate_system_orientation</t>
   </si>
   <si>
-    <t>"nozzle_to_combustion_chamber"</t>
-  </si>
-  <si>
     <t>dry_inertia_i11</t>
   </si>
   <si>
@@ -143,9 +137,6 @@
     <t>tuple</t>
   </si>
   <si>
-    <t>"tail_to_nose"</t>
-  </si>
-  <si>
     <t>kg</t>
   </si>
   <si>
@@ -237,6 +228,57 @@
   </si>
   <si>
     <t>angular_position</t>
+  </si>
+  <si>
+    <t>motor_radius</t>
+  </si>
+  <si>
+    <t>diameter98mm</t>
+  </si>
+  <si>
+    <t>Supprt Vars</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>nozzle_to_combustion_chamber</t>
+  </si>
+  <si>
+    <t>AeroTech_M1939W.eng</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>latitude</t>
+  </si>
+  <si>
+    <t>longitude</t>
+  </si>
+  <si>
+    <t>elevation</t>
+  </si>
+  <si>
+    <t>standard_atmosphere</t>
+  </si>
+  <si>
+    <t>tail_to_nose</t>
+  </si>
+  <si>
+    <t>atmospheric_model</t>
   </si>
 </sst>
 </file>
@@ -295,6 +337,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6299667B-1921-474E-B0A2-56EDAD39ED1B}" name="Table1" displayName="Table1" ref="A1:D23" totalsRowShown="0">
+  <autoFilter ref="A1:D23" xr:uid="{6299667B-1921-474E-B0A2-56EDAD39ED1B}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{DF57E6C4-8BD4-41F9-B65D-B0A3EFA0455B}" name="Variable"/>
+    <tableColumn id="2" xr3:uid="{4EE4F1BB-B34D-4DB8-AB26-2281CC688B45}" name="Set"/>
+    <tableColumn id="3" xr3:uid="{1CD5815B-3688-4DC4-9B7A-828E32A42543}" name="Column1"/>
+    <tableColumn id="4" xr3:uid="{9CF19FE7-F57C-4590-8616-EB2FE2A6693C}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -614,255 +669,371 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0D88883-570E-48D5-9EA0-8E8B677054BE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8160EB66-A072-414B-B1B5-A2EF0AE3FFBA}">
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
       <c r="D1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2">
+        <f>98/2/25.4</f>
+        <v>1.9291338582677167</v>
+      </c>
+      <c r="I2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
       </c>
       <c r="B3">
         <f>(1.75/2) / 39.37</f>
         <v>2.2225044450088903E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B4">
         <v>3.2690000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5">
+        <f>(1/12)*B4*(3*((G2*2)+POWER(0.732,2)))</f>
+        <v>3.5910714553385823</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>21</v>
       </c>
-      <c r="B5">
-        <f>(1/12)*B4*(3*((0.098/2)*2)+POWER(0.732,2))</f>
-        <v>0.22605788799999998</v>
-      </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
       <c r="B6">
-        <f>(1/12)*B4*(3*((0.098/2)*2)+POWER(0.732,2))</f>
-        <v>0.22605788799999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+        <f>(1/12)*B4*(3*((G2)*2)+POWER(0.732,2))</f>
+        <v>3.2991366793385826</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B7">
-        <f>0.5*B4*POWER((0.098/2),2)</f>
-        <v>3.9244345000000007E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+        <f>0.5*B4*POWER((G2),2)</f>
+        <v>6.0828856407712824</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <f>0.06576*27679.90471</f>
         <v>1820.2305337296</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <f>3.365/2/39.37</f>
         <v>4.2735585471170949E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <f>1.125/2/39.37</f>
         <v>1.428752857505715E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <f>6/2/39.37</f>
         <v>7.620015240030481E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <f>6/2/39.37/2</f>
         <v>3.8100076200152405E-2</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <f>0.732/2</f>
         <v>0.36599999999999999</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>6.2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <f>0.734/2/39.37</f>
         <v>9.3218186436372884E-3</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19">
+        <v>212</v>
+      </c>
+      <c r="D19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20">
+        <v>21</v>
+      </c>
+      <c r="D20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>54</v>
       </c>
-      <c r="D19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>57</v>
+      <c r="B22">
+        <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>55</v>
+      </c>
+      <c r="B23">
+        <v>21</v>
       </c>
       <c r="D23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DE46F10-F7E4-4FF9-9DF9-CA245AB9C3B3}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -879,21 +1050,21 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <f>6.17/2/39.37</f>
         <v>7.8359156718313436E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -905,38 +1076,38 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>26</v>
       </c>
-      <c r="G4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -947,14 +1118,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D4D93E-62F8-4675-8413-8C8F2B28BDDF}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="11" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -971,60 +1142,60 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="G5" t="s">
         <v>47</v>
       </c>
-      <c r="G4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" t="s">
         <v>48</v>
-      </c>
-      <c r="G7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1035,12 +1206,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C6CA8B0-88A8-433F-A0FC-EB53EF89F6DB}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1057,63 +1228,63 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B2">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>43</v>
       </c>
       <c r="B6">
         <f>6.17/2/39.37</f>
         <v>7.8359156718313436E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1124,12 +1295,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C24AA439-E62A-4D19-BE31-DD01D82FC1DB}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1146,40 +1317,40 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" t="s">
         <v>49</v>
-      </c>
-      <c r="G7" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1190,9 +1361,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B40BE1E-2C0B-4286-A3FB-3C7826FF8F5E}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1209,27 +1380,27 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
it works i think 1. fixed input errors 2. numpy.arange so range can include floats 2. created single sim function 3. all nested for loops 4. concurrency 5. output file 6. not fully tested, i have it as file appened at the end of the program. 7. need to fix fin flutter analysis
</commit_message>
<xml_diff>
--- a/rpy_input_parameters.xlsx
+++ b/rpy_input_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samjo\Desktop\clubs\soar\irec_27\controls_eecs\IREC_26-27_Controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A6356C-3C7C-4424-9938-772D6081D2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E471B4A8-A96A-4040-99AC-D6FB38496F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{3850124B-4C10-4519-AB6D-3AC4B4A0B5D5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="2" activeTab="4" xr2:uid="{3850124B-4C10-4519-AB6D-3AC4B4A0B5D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Environment" sheetId="2" r:id="rId1"/>
@@ -18,8 +18,10 @@
     <sheet name="Rocket" sheetId="3" r:id="rId3"/>
     <sheet name="Nosecone" sheetId="4" r:id="rId4"/>
     <sheet name="Trapezoidal Fins" sheetId="5" r:id="rId5"/>
-    <sheet name="Tail" sheetId="6" r:id="rId6"/>
-    <sheet name="Rail Buttons" sheetId="7" r:id="rId7"/>
+    <sheet name="Rail Buttons" sheetId="7" r:id="rId6"/>
+    <sheet name="Flight" sheetId="9" r:id="rId7"/>
+    <sheet name="Post Flight Filters" sheetId="10" r:id="rId8"/>
+    <sheet name="Pre Flight Filters" sheetId="11" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="144">
   <si>
     <t>Variable</t>
   </si>
@@ -119,9 +121,6 @@
     <t>mass</t>
   </si>
   <si>
-    <t>inertia</t>
-  </si>
-  <si>
     <t>power_off_drag</t>
   </si>
   <si>
@@ -131,161 +130,362 @@
     <t>center_of_mass_without_motor</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>tuple</t>
   </si>
   <si>
-    <t>kg</t>
-  </si>
-  <si>
     <t>length</t>
   </si>
   <si>
+    <t>kind</t>
+  </si>
+  <si>
+    <t>bluffness</t>
+  </si>
+  <si>
+    <t>ogive</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>root_chord</t>
+  </si>
+  <si>
+    <t>tip_chord</t>
+  </si>
+  <si>
+    <t>span</t>
+  </si>
+  <si>
+    <t>sweep_length</t>
+  </si>
+  <si>
+    <t>sweep_angle</t>
+  </si>
+  <si>
+    <t>airfoil</t>
+  </si>
+  <si>
+    <t>base_radius</t>
+  </si>
+  <si>
+    <t>power</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>optional/no impact</t>
+  </si>
+  <si>
+    <t>optional</t>
+  </si>
+  <si>
+    <t>dry_mass</t>
+  </si>
+  <si>
+    <t>reshape_thrust_curve</t>
+  </si>
+  <si>
+    <t>no idea</t>
+  </si>
+  <si>
+    <t>interpolation_method</t>
+  </si>
+  <si>
+    <t>reference_pressure</t>
+  </si>
+  <si>
+    <t>only_radial_burn</t>
+  </si>
+  <si>
+    <t>upper_button_position</t>
+  </si>
+  <si>
+    <t>lower_button_position</t>
+  </si>
+  <si>
+    <t>angular_position</t>
+  </si>
+  <si>
+    <t>motor_radius</t>
+  </si>
+  <si>
+    <t>diameter98mm</t>
+  </si>
+  <si>
+    <t>Supprt Vars</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>nozzle_to_combustion_chamber</t>
+  </si>
+  <si>
+    <t>AeroTech_M1939W.eng</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>latitude</t>
+  </si>
+  <si>
+    <t>longitude</t>
+  </si>
+  <si>
+    <t>elevation</t>
+  </si>
+  <si>
+    <t>standard_atmosphere</t>
+  </si>
+  <si>
+    <t>tail_to_nose</t>
+  </si>
+  <si>
+    <t>atmospheric_model</t>
+  </si>
+  <si>
+    <t>kg, mass without motor</t>
+  </si>
+  <si>
+    <t>rocket dry inertia tensor</t>
+  </si>
+  <si>
+    <t>inertia_i11</t>
+  </si>
+  <si>
+    <t>inertia_i22</t>
+  </si>
+  <si>
+    <t>inertia_i33</t>
+  </si>
+  <si>
     <t>position</t>
   </si>
   <si>
-    <t>kind</t>
-  </si>
-  <si>
-    <t>bluffness</t>
-  </si>
-  <si>
-    <t>ogive</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>root_chord</t>
-  </si>
-  <si>
-    <t>tip_chord</t>
-  </si>
-  <si>
-    <t>span</t>
-  </si>
-  <si>
-    <t>rocket_radius</t>
-  </si>
-  <si>
-    <t>sweep_length</t>
-  </si>
-  <si>
-    <t>sweep_angle</t>
-  </si>
-  <si>
-    <t>airfoil</t>
-  </si>
-  <si>
-    <t>base_radius</t>
-  </si>
-  <si>
-    <t>power</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>needed for ogive</t>
-  </si>
-  <si>
-    <t>optional/no impact</t>
-  </si>
-  <si>
-    <t>optional</t>
-  </si>
-  <si>
-    <t>dry_mass</t>
-  </si>
-  <si>
-    <t>reshape_thrust_curve</t>
-  </si>
-  <si>
-    <t>no idea</t>
-  </si>
-  <si>
-    <t>interpolation_method</t>
-  </si>
-  <si>
-    <t>reference_pressure</t>
-  </si>
-  <si>
-    <t>only_radial_burn</t>
-  </si>
-  <si>
-    <t>top_radius</t>
-  </si>
-  <si>
-    <t>bottom_radius</t>
-  </si>
-  <si>
-    <t>upper_button_position</t>
-  </si>
-  <si>
-    <t>lower_button_position</t>
-  </si>
-  <si>
-    <t>angular_position</t>
-  </si>
-  <si>
-    <t>motor_radius</t>
-  </si>
-  <si>
-    <t>diameter98mm</t>
-  </si>
-  <si>
-    <t>Supprt Vars</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>nozzle_to_combustion_chamber</t>
-  </si>
-  <si>
-    <t>AeroTech_M1939W.eng</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>day</t>
-  </si>
-  <si>
-    <t>hour</t>
-  </si>
-  <si>
-    <t>latitude</t>
-  </si>
-  <si>
-    <t>longitude</t>
-  </si>
-  <si>
-    <t>elevation</t>
-  </si>
-  <si>
-    <t>standard_atmosphere</t>
-  </si>
-  <si>
-    <t>tail_to_nose</t>
-  </si>
-  <si>
-    <t>atmospheric_model</t>
+    <t>optional, needed for powerseries, factor that controls bluntess of nose cone shape</t>
+  </si>
+  <si>
+    <t>optional, if not given then default is rocket radius</t>
+  </si>
+  <si>
+    <t>von karman, conical, ogive, ivhaac, and powerseries</t>
+  </si>
+  <si>
+    <t>https://docs.rocketpy.org/en/latest/user/positions.html#:~:text=the%20coordinate%20system%20origin%20and%20orientation.-,Example,-with%20Origin%20at%20Arbitrary%20Point%23</t>
+  </si>
+  <si>
+    <t>based off of rocket.coordinate system orientation</t>
+  </si>
+  <si>
+    <t>Notes, https://docs.rocketpy.org/en/latest/reference/classes/Rocket.html#rocketpy.Rocket.add_nose:~:text=Tail-,add_nose,-(length%2C</t>
+  </si>
+  <si>
+    <t>Notes, https://docs.rocketpy.org/en/latest/reference/classes/Rocket.html#rocketpy.Rocket.add_nose:~:text=kg*m%5E2.-,__init__,-(radius%2C</t>
+  </si>
+  <si>
+    <t>Notes, https://docs.rocketpy.org/en/latest/reference/classes/Rocket.html#rocketpy.Rocket.add_nose:~:text=arguments%20and%20signature.-,add_trapezoidal_fins,-(n%2C</t>
+  </si>
+  <si>
+    <t>cant_angle</t>
+  </si>
+  <si>
+    <t>based on rocket coordinate system</t>
+  </si>
+  <si>
+    <t>Notes, https://docs.rocketpy.org/en/latest/reference/classes/Rocket.html#rocketpy.Rocket.add_nose:~:text=Controller%20object%20created.-,set_rail_buttons,-(upper_button_position%2C</t>
+  </si>
+  <si>
+    <t>Notes, https://docs.rocketpy.org/en/latest/reference/classes/motors/SolidMotor.html#:~:text=Default%20is%20False.-,__init__,-(thrust_source%2C</t>
+  </si>
+  <si>
+    <t>SRAD Nosecone</t>
+  </si>
+  <si>
+    <t>tecnically optional, but needed for ogive, ratio between radius of circle on tip of ogive and radius of base, programable with this variable meaning radius of tip</t>
+  </si>
+  <si>
+    <t>fin count</t>
+  </si>
+  <si>
+    <t>rocket</t>
+  </si>
+  <si>
+    <t>nika</t>
+  </si>
+  <si>
+    <t>environment</t>
+  </si>
+  <si>
+    <t>env</t>
+  </si>
+  <si>
+    <t>rail_length</t>
+  </si>
+  <si>
+    <t>inclination</t>
+  </si>
+  <si>
+    <t>Notes, https://docs.rocketpy.org/en/latest/reference/classes/Flight.html#:~:text=phase%20in%20N%C2%B7m.-,__init__,-(rocket%2C</t>
+  </si>
+  <si>
+    <t>optional, angle relative to ground</t>
+  </si>
+  <si>
+    <t>heading</t>
+  </si>
+  <si>
+    <t>initial_solution</t>
+  </si>
+  <si>
+    <t>optional, uses previous state if we have it</t>
+  </si>
+  <si>
+    <t>optional, heading angle, which I think is based off of inclination</t>
+  </si>
+  <si>
+    <t>terminate_on_apogee</t>
+  </si>
+  <si>
+    <t>optional, stop sim after rocket reaches apogee.</t>
+  </si>
+  <si>
+    <t>max_time</t>
+  </si>
+  <si>
+    <t>optional, seconds, default is 600</t>
+  </si>
+  <si>
+    <t>max_time_step</t>
+  </si>
+  <si>
+    <t>optional, default is .01. needed if max_time is chaged</t>
+  </si>
+  <si>
+    <t>min_time_step</t>
+  </si>
+  <si>
+    <t>rtol</t>
+  </si>
+  <si>
+    <t>optional, max relative error to be tolerated in integration scheme</t>
+  </si>
+  <si>
+    <t>atol</t>
+  </si>
+  <si>
+    <t>optional, max absolute error to be tolerated in integration scheme</t>
+  </si>
+  <si>
+    <t>optional, this and above row has most impact on time to complete simulation</t>
+  </si>
+  <si>
+    <t>time_overshoot</t>
+  </si>
+  <si>
+    <t>optional, I think meant for parachutes</t>
+  </si>
+  <si>
+    <t>verbose</t>
+  </si>
+  <si>
+    <t>equations_of_motion</t>
+  </si>
+  <si>
+    <t>solid_propulsion</t>
+  </si>
+  <si>
+    <t>optional, defualt is standard</t>
+  </si>
+  <si>
+    <t>ode_solver</t>
+  </si>
+  <si>
+    <t>optional, integration methodto sove EoM</t>
+  </si>
+  <si>
+    <t>simulation_mode</t>
+  </si>
+  <si>
+    <t>6 DOF</t>
+  </si>
+  <si>
+    <t>optional., default is 6 dof</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>optional, Angular position of the rail buttons in degrees measured as the rotation around the symmetry axis of the rocket relative to one of the other principal axis. Default value is 45 degrees, generally used in rockets with 4</t>
+  </si>
+  <si>
+    <t>button furtherst from nozzle</t>
+  </si>
+  <si>
+    <t>button closest from nozzle</t>
+  </si>
+  <si>
+    <t>optional, reference radius of rocket</t>
+  </si>
+  <si>
+    <t>optional, fuselage radius</t>
+  </si>
+  <si>
+    <t>Operator</t>
+  </si>
+  <si>
+    <t>Threshold</t>
+  </si>
+  <si>
+    <t>&lt;=</t>
+  </si>
+  <si>
+    <t>Notes: removes the flight</t>
+  </si>
+  <si>
+    <t>if apogee is less than 10500feet, cut</t>
+  </si>
+  <si>
+    <t>apogee</t>
+  </si>
+  <si>
+    <t>&gt;=</t>
+  </si>
+  <si>
+    <t>max_mach_number</t>
+  </si>
+  <si>
+    <t>fin_thickness</t>
+  </si>
+  <si>
+    <t>shear_modulus</t>
+  </si>
+  <si>
+    <t>for flutter analysis, in Pascals</t>
+  </si>
+  <si>
+    <t>for flutter analysis, https://docs.rocketpy.org/en/latest/reference/classes/utils/utilities.html#rocketpy.utilities.liftoff_speed_by_mass:~:text=rocketpy.utilities.-,fin_flutter_analysis,-(fin_thickness%2C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +495,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -317,13 +525,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -346,7 +557,7 @@
     <tableColumn id="1" xr3:uid="{DF57E6C4-8BD4-41F9-B65D-B0A3EFA0455B}" name="Variable"/>
     <tableColumn id="2" xr3:uid="{4EE4F1BB-B34D-4DB8-AB26-2281CC688B45}" name="Set"/>
     <tableColumn id="3" xr3:uid="{1CD5815B-3688-4DC4-9B7A-828E32A42543}" name="Column1"/>
-    <tableColumn id="4" xr3:uid="{9CF19FE7-F57C-4590-8616-EB2FE2A6693C}" name="Notes"/>
+    <tableColumn id="4" xr3:uid="{9CF19FE7-F57C-4590-8616-EB2FE2A6693C}" name="Notes, https://docs.rocketpy.org/en/latest/reference/classes/motors/SolidMotor.html#:~:text=Default%20is%20False.-,__init__,-(thrust_source%2C"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -670,13 +881,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0D88883-570E-48D5-9EA0-8E8B677054BE}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -684,68 +895,68 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B2">
         <v>2027</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B3">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B4">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B5">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -756,18 +967,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8160EB66-A072-414B-B1B5-A2EF0AE3FFBA}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -775,37 +986,37 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="G1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G2">
         <f>98/2/25.4</f>
         <v>1.9291338582677167</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -814,15 +1025,15 @@
         <v>2.2225044450088903E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B4">
         <v>3.2690000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -831,10 +1042,10 @@
         <v>3.5910714553385823</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -843,7 +1054,7 @@
         <v>3.2991366793385826</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -852,7 +1063,7 @@
         <v>6.0828856407712824</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -860,7 +1071,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -869,7 +1080,7 @@
         <v>1820.2305337296</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -878,7 +1089,7 @@
         <v>4.2735585471170949E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -887,7 +1098,7 @@
         <v>1.428752857505715E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -896,7 +1107,7 @@
         <v>7.620015240030481E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -904,7 +1115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -913,10 +1124,10 @@
         <v>3.8100076200152405E-2</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -925,10 +1136,10 @@
         <v>0.36599999999999999</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -936,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -947,7 +1158,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -956,62 +1167,62 @@
         <v>9.3218186436372884E-3</v>
       </c>
       <c r="D18" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B19">
         <v>212</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B20">
         <v>21</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D21" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B22">
         <v>21</v>
       </c>
       <c r="D22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>55</v>
       </c>
       <c r="B23">
         <v>21</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1026,14 +1237,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DE46F10-F7E4-4FF9-9DF9-CA245AB9C3B3}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1050,10 +1262,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1062,7 +1274,7 @@
         <v>7.8359156718313436E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1076,56 +1288,92 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>24</v>
       </c>
-      <c r="G4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B8">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
-        <v>76</v>
+      <c r="B10" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="G10" r:id="rId1" location=":~:text=the%20coordinate%20system%20origin%20and%20orientation.-,Example,-with%20Origin%20at%20Arbitrary%20Point%23" xr:uid="{DE2AC066-B816-467E-8B6C-2D9FE5019A1E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D4D93E-62F8-4675-8413-8C8F2B28BDDF}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="11" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11" customWidth="1"/>
+    <col min="7" max="7" width="137.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1142,60 +1390,106 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="D3">
+        <f>10/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="G3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>75</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>30</v>
+      </c>
+      <c r="C5">
+        <v>0.1</v>
+      </c>
+      <c r="D5">
+        <v>0.9</v>
+      </c>
+      <c r="E5">
+        <v>0.1</v>
       </c>
       <c r="G5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>40</v>
       </c>
+      <c r="B6" t="s">
+        <v>126</v>
+      </c>
       <c r="G6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>88</v>
       </c>
       <c r="G7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>126</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1205,13 +1499,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C6CA8B0-88A8-433F-A0FC-EB53EF89F6DB}">
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="143" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1228,63 +1523,166 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B2">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3">
+        <v>0.5</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>0.5</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5">
+        <v>0.5</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6">
+        <v>0.5</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>0.1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7">
+        <v>0.5</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0.1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8">
+        <v>0.5</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>0.1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B9" t="s">
+        <v>126</v>
+      </c>
+      <c r="G9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>0.2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6">
-        <f>6.17/2/39.37</f>
-        <v>7.8359156718313436E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B11" t="s">
+        <v>126</v>
+      </c>
+      <c r="G11" t="s">
         <v>43</v>
       </c>
-      <c r="G9" t="s">
-        <v>49</v>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B12">
+        <v>0.25</v>
+      </c>
+      <c r="G12" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13">
+        <v>0.4</v>
+      </c>
+      <c r="G13" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1293,14 +1691,15 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C24AA439-E62A-4D19-BE31-DD01D82FC1DB}">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B40BE1E-2C0B-4286-A3FB-3C7826FF8F5E}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="156.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1317,40 +1716,63 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="C2">
+        <v>0.5</v>
+      </c>
+      <c r="D2">
+        <v>0.8</v>
+      </c>
+      <c r="E2">
+        <v>0.1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="C3">
+        <v>0.4</v>
+      </c>
+      <c r="D3">
+        <v>0.7</v>
+      </c>
+      <c r="E3">
+        <v>0.1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="B4">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
+      <c r="B5">
+        <v>0.1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1359,11 +1781,16 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B40BE1E-2C0B-4286-A3FB-3C7826FF8F5E}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7BEC39-01EF-4B9C-8864-8478383F670F}">
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="119.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1380,30 +1807,273 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="B3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>12</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>96</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9">
+        <v>500</v>
+      </c>
+      <c r="G9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10">
+        <v>0.01</v>
+      </c>
+      <c r="G10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11">
+        <v>0.01</v>
+      </c>
+      <c r="G11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>126</v>
+      </c>
+      <c r="G12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G13" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>117</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" t="s">
+        <v>126</v>
+      </c>
+      <c r="G17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" t="s">
+        <v>124</v>
+      </c>
+      <c r="G18" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970CA711-3322-4827-896D-9B272721D0E5}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2">
+        <v>10500</v>
+      </c>
+      <c r="E2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4">
+        <v>0.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08DD3E74-9FB8-42C9-816D-A1DFF162828F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>